<commit_message>
Bulkupload fixes in content generations
</commit_message>
<xml_diff>
--- a/bulk_content_upload_template.xlsx
+++ b/bulk_content_upload_template.xlsx
@@ -21,6 +21,10 @@
     <definedName name="TargetLanguages">'_Lookup'!$H$2:$H$10</definedName>
     <definedName name="TargetAudiences">'_Lookup'!$I$2:$I$5</definedName>
     <definedName name="Priorities">'_Lookup'!$M$2:$M$4</definedName>
+    <definedName name="WC_Social_Media">'_Lookup'!$J$2:$J$5</definedName>
+    <definedName name="WC_Community">'_Lookup'!$K$2:$K$5</definedName>
+    <definedName name="WC_Articles">'_Lookup'!$L$2:$L$6</definedName>
+    <definedName name="WC_Web_Pages">'_Lookup'!$L$2:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bulk Upload'!$A$1:$P$501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9937,8 +9941,8 @@
     <dataValidation sqref="G2:G501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Audience" error="Please select from: General, Beginners, Professionals, Experts" promptTitle="Target Audience" prompt="Select the target audience level" type="list">
       <formula1>TargetAudiences</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Word Count" error="Please select a valid word count: 50,150,300,400,500,800,1500,2000,2500,3500" promptTitle="Word Count" prompt="Social Media: 50-500 | Community: 150-1500 | Articles/Pages: 800-3500" type="list">
-      <formula1>"50,150,300,400,500,800,1500,2000,2500,3500"</formula1>
+    <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Word Count" error="Please first select a Content Category in column A, then choose a valid Word Count for that category. Articles/Web Pages: 800-3500 | Social Media: 50-500 | Community: 150-1500" promptTitle="Word Count" prompt="First select Content Category (column A), then pick a Word Count valid for that category. Articles/Web Pages: 800-3500 | Social Media: 50-500 | Community: 150-1500" type="list">
+      <formula1>=INDIRECT("WC_"&amp;SUBSTITUTE(A2," ","_"))</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Priority" error="Please select from: High, Medium, Low" promptTitle="Priority" prompt="Select the content priority level" type="list">
       <formula1>Priorities</formula1>
@@ -10627,7 +10631,7 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Dropdown: Social Media(50-500) | Community(150-1500) | Articles/Pages(800-3500)</t>
+          <t>Cascading Dropdown: Options change based on Content Category. Articles/Web Pages: 800-3500 | Social Media: 50-500 | Community: 150-1500</t>
         </is>
       </c>
     </row>

</xml_diff>